<commit_message>
LambdaMapping - backtest to StrategyBase.xlsx: added stage_strat_specific_preentry_data
</commit_message>
<xml_diff>
--- a/siglab_py/LambdaMapping - backtest to StrategyBase.xlsx
+++ b/siglab_py/LambdaMapping - backtest to StrategyBase.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29426"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\dev\siglab\siglab_py\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{18612270-CF21-4B60-97A8-15EF959E37D0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{121A4409-8AB1-4E41-AA0A-991A76FDBB9F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-17100" yWindow="-170" windowWidth="12110" windowHeight="8375" xr2:uid="{64FB003A-71C9-4620-8FE1-FA72144932C7}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{64FB003A-71C9-4620-8FE1-FA72144932C7}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="18" uniqueCount="13">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="20" uniqueCount="14">
   <si>
     <t>allow_entry_initial</t>
   </si>
@@ -75,6 +75,9 @@
   </si>
   <si>
     <t>allow_entry_init</t>
+  </si>
+  <si>
+    <t>stage_strat_specific_preentry_data</t>
   </si>
 </sst>
 </file>
@@ -469,11 +472,11 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6C1637B9-DBB5-4545-BBD1-03BE4CC4FC5A}">
-  <dimension ref="A1:C9"/>
+  <dimension ref="A1:C10"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="2" bestFit="1" customWidth="1"/>
-    <col min="2" max="3" width="23.5546875" bestFit="1" customWidth="1"/>
+    <col min="2" max="3" width="29.109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:3" s="1" customFormat="1" x14ac:dyDescent="0.3">
@@ -572,6 +575,17 @@
         <v>9</v>
       </c>
     </row>
+    <row r="10" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A10">
+        <v>9</v>
+      </c>
+      <c r="B10" t="s">
+        <v>13</v>
+      </c>
+      <c r="C10" t="s">
+        <v>13</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>

</xml_diff>